<commit_message>
Stage 8 review fixes: F-008
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/Development/AU08/Vehicle_Ladder/Bench_Sheets/AU08_vehicle-ladder_051316_MS.xlsx
+++ b/output/archive/DurnesswickData/Development/AU08/Vehicle_Ladder/Bench_Sheets/AU08_vehicle-ladder_051316_MS.xlsx
@@ -649,7 +649,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Vehicle screen (table of 8 vehicles), Recipe card (buffer-adjusted solution), Notes</t>
+          <t>Vehicle screen, Recipe card, Notes</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -923,123 +923,43 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Selected for exposure work. Pilot lot scale is not yet agreed with the client.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Selected for exposure work; selection does not establish a locked scale process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Refer to the source recipe card for buffer identity, pH, excipient levels and preparation sequence.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Dilution outcome</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Basis</t>
+          <t>Buffer adjustment prevented precipitation on dilution. Refer to the dilution bench record for conditions and observations.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Active (AU-08)</t>
+          <t>Screen limitation</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Model compound</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Target 10 mg/mL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Citrate buffer</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>pH control</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Buffer adjustment prevented precipitation on dilution</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Solubilising cosolvent</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Solubility aid</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Kept at the lowest level that held the solution clear</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Preservative</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Microbial control</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Per client excipient list</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Flavour and sweetener</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Palatability</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Deferred to the client's paediatric panel</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Note for the pilot lot</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>The unbuffered recipe precipitated on dilution. Do not drop the buffer step when scaling.</t>
+          <t>The initial vehicle screen is separate from the adjusted recipe. Clarity at preparation alone did not establish physical stability.</t>
         </is>
       </c>
     </row>
@@ -1056,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1083,31 +1003,19 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Interim read: the cosolvent-rich recipes held at 10 mg/mL but grew crystals within 24 h. Buffer adjustment looks like the fix; dilution photos go in the readout.</t>
+          <t>Initial screen: Labrasol/PEG400 was clear at preparation but precipitated at 24 h. Other vehicles were suspensions; their physical behavior is recorded in the vehicle screen.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>05/24/2016</t>
+          <t>06/06/2016</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Excipient compatibility repeat run on the buffered recipe. No colour change. Screen suitability checks passed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>06/06/2016</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Final bench sheet. Readout DL_2016_0027 issued the same day. Recipe card locked for the exposure work.</t>
+          <t>Buffer adjustment prevented precipitation on dilution and Auvrelquith selected the solution for exposure work. The source recipe card carries preparation details.</t>
         </is>
       </c>
     </row>

</xml_diff>